<commit_message>
pbi validator and other feature enhancements
</commit_message>
<xml_diff>
--- a/output/Test_Cases_collection/---.xlsx
+++ b/output/Test_Cases_collection/---.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,348 +525,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>---:</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>---</t>
+          <t>---:</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>---:</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
         <is>
           <t>---</t>
         </is>

</xml_diff>